<commit_message>
Strengthen survey QA and output reconciliation
</commit_message>
<xml_diff>
--- a/output/tab_books/Reach3_Social_Media_TabBook.xlsx
+++ b/output/tab_books/Reach3_Social_Media_TabBook.xlsx
@@ -17,7 +17,7 @@
     <sheet name="08_QA_SUMMARY" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'08_QA_SUMMARY'!$A$1:$K$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'08_QA_SUMMARY'!$A$1:$P$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18551,7 +18551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18563,8 +18563,13 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="38" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18595,30 +18600,55 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
+          <t>substantive_response_n</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
           <t>valid_n</t>
         </is>
       </c>
-      <c r="G1" s="18" t="inlineStr">
-        <is>
-          <t>special_or_invalid_n</t>
-        </is>
-      </c>
       <c r="H1" s="18" t="inlineStr">
         <is>
+          <t>special_99_n</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>missing_outcome_n</t>
+        </is>
+      </c>
+      <c r="J1" s="18" t="inlineStr">
+        <is>
+          <t>unexpected_response_n</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="inlineStr">
+        <is>
+          <t>missing_weight_n</t>
+        </is>
+      </c>
+      <c r="L1" s="18" t="inlineStr">
+        <is>
+          <t>invalid_weight_n</t>
+        </is>
+      </c>
+      <c r="M1" s="18" t="inlineStr">
+        <is>
           <t>weighted_base</t>
         </is>
       </c>
-      <c r="I1" s="18" t="inlineStr">
+      <c r="N1" s="18" t="inlineStr">
         <is>
           <t>percentage_qa</t>
         </is>
       </c>
-      <c r="J1" s="18" t="inlineStr">
+      <c r="O1" s="18" t="inlineStr">
         <is>
           <t>measure</t>
         </is>
       </c>
-      <c r="K1" s="18" t="inlineStr">
+      <c r="P1" s="18" t="inlineStr">
         <is>
           <t>universe</t>
         </is>
@@ -18652,22 +18682,37 @@
         <v>7135</v>
       </c>
       <c r="G2" s="4" t="n">
+        <v>7135</v>
+      </c>
+      <c r="H2" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="4" t="n">
         <v>7236.64294794</v>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Get news</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKFB_W144 == 1</t>
         </is>
@@ -18701,22 +18746,37 @@
         <v>7136</v>
       </c>
       <c r="G3" s="4" t="n">
+        <v>7136</v>
+      </c>
+      <c r="H3" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
         <v>7244.06282044</v>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Keep up with politics or political issues</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKFB_W144 == 1</t>
         </is>
@@ -18750,22 +18810,37 @@
         <v>7139</v>
       </c>
       <c r="G4" s="4" t="n">
+        <v>7139</v>
+      </c>
+      <c r="H4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>7245.88148694</v>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Keep up with sports or pop culture</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKFB_W144 == 1</t>
         </is>
@@ -18799,22 +18874,37 @@
         <v>7142</v>
       </c>
       <c r="G5" s="4" t="n">
+        <v>7142</v>
+      </c>
+      <c r="H5" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="4" t="n">
         <v>7250.02123249</v>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>Entertainment</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKFB_W144 == 1</t>
         </is>
@@ -18848,22 +18938,37 @@
         <v>7144</v>
       </c>
       <c r="G6" s="4" t="n">
+        <v>7144</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>7250.85933721</v>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Keep up with friends and family</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKFB_W144 == 1</t>
         </is>
@@ -18897,22 +19002,37 @@
         <v>7140</v>
       </c>
       <c r="G7" s="4" t="n">
+        <v>7140</v>
+      </c>
+      <c r="H7" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4" t="n">
         <v>7242.50945524</v>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>Connect with others who share your interests</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKFB_W144 == 1</t>
         </is>
@@ -18946,22 +19066,37 @@
         <v>7143</v>
       </c>
       <c r="G8" s="4" t="n">
+        <v>7143</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>7245.41661774</v>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Look at product reviews or recommendations</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKFB_W144 == 1</t>
         </is>
@@ -18995,22 +19130,37 @@
         <v>4489</v>
       </c>
       <c r="G9" s="4" t="n">
+        <v>4489</v>
+      </c>
+      <c r="H9" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4" t="n">
         <v>5171.96307175</v>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>Get news</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKIG_W144 == 1</t>
         </is>
@@ -19044,22 +19194,37 @@
         <v>4497</v>
       </c>
       <c r="G10" s="4" t="n">
+        <v>4497</v>
+      </c>
+      <c r="H10" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>5172.22195928</v>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Keep up with politics or political issues</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKIG_W144 == 1</t>
         </is>
@@ -19093,22 +19258,37 @@
         <v>4496</v>
       </c>
       <c r="G11" s="4" t="n">
+        <v>4496</v>
+      </c>
+      <c r="H11" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="4" t="n">
         <v>5166.07800467</v>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>Keep up with sports or pop culture</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="P11" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKIG_W144 == 1</t>
         </is>
@@ -19142,22 +19322,37 @@
         <v>4496</v>
       </c>
       <c r="G12" s="4" t="n">
+        <v>4496</v>
+      </c>
+      <c r="H12" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>5172.35712365</v>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>Entertainment</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKIG_W144 == 1</t>
         </is>
@@ -19191,22 +19386,37 @@
         <v>4501</v>
       </c>
       <c r="G13" s="4" t="n">
+        <v>4501</v>
+      </c>
+      <c r="H13" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="I13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="4" t="n">
         <v>5175.4740633</v>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>Keep up with friends and family</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKIG_W144 == 1</t>
         </is>
@@ -19240,22 +19450,37 @@
         <v>4492</v>
       </c>
       <c r="G14" s="4" t="n">
+        <v>4492</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>5164.15428303</v>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>Connect with others who share your interests</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKIG_W144 == 1</t>
         </is>
@@ -19289,22 +19514,37 @@
         <v>4501</v>
       </c>
       <c r="G15" s="4" t="n">
+        <v>4501</v>
+      </c>
+      <c r="H15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="4" t="n">
         <v>5181.73182042</v>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>Look at product reviews or recommendations</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>DOV_ASKIG_W144 == 1</t>
         </is>
@@ -19338,22 +19578,37 @@
         <v>2555</v>
       </c>
       <c r="G16" s="4" t="n">
+        <v>2555</v>
+      </c>
+      <c r="H16" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="4" t="n">
         <v>2570.90942585</v>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Get news</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>SMUSE_c_W144 == 1</t>
         </is>
@@ -19387,22 +19642,37 @@
         <v>2554</v>
       </c>
       <c r="G17" s="4" t="n">
+        <v>2554</v>
+      </c>
+      <c r="H17" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="4" t="n">
         <v>2570.64721703</v>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>Keep up with politics or political issues</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="P17" s="4" t="inlineStr">
         <is>
           <t>SMUSE_c_W144 == 1</t>
         </is>
@@ -19436,22 +19706,37 @@
         <v>2555</v>
       </c>
       <c r="G18" s="4" t="n">
+        <v>2555</v>
+      </c>
+      <c r="H18" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="4" t="n">
         <v>2570.44580276</v>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>Keep up with sports or pop culture</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>SMUSE_c_W144 == 1</t>
         </is>
@@ -19485,22 +19770,37 @@
         <v>2551</v>
       </c>
       <c r="G19" s="4" t="n">
+        <v>2551</v>
+      </c>
+      <c r="H19" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H19" s="4" t="n">
+      <c r="I19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="4" t="n">
         <v>2571.3851121</v>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>Entertainment</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="P19" s="4" t="inlineStr">
         <is>
           <t>SMUSE_c_W144 == 1</t>
         </is>
@@ -19534,22 +19834,37 @@
         <v>2557</v>
       </c>
       <c r="G20" s="4" t="n">
+        <v>2557</v>
+      </c>
+      <c r="H20" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="I20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="4" t="n">
         <v>2567.34400811</v>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>Keep up with friends and family</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>SMUSE_c_W144 == 1</t>
         </is>
@@ -19583,22 +19898,37 @@
         <v>2557</v>
       </c>
       <c r="G21" s="4" t="n">
+        <v>2557</v>
+      </c>
+      <c r="H21" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="I21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="4" t="n">
         <v>2577.00314592</v>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>Connect with others who share your interests</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="P21" s="4" t="inlineStr">
         <is>
           <t>SMUSE_c_W144 == 1</t>
         </is>
@@ -19632,22 +19962,37 @@
         <v>2557</v>
       </c>
       <c r="G22" s="4" t="n">
+        <v>2557</v>
+      </c>
+      <c r="H22" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="I22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="4" t="n">
         <v>2572.09326106</v>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>Look at product reviews or recommendations</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>SMUSE_c_W144 == 1</t>
         </is>
@@ -19681,22 +20026,37 @@
         <v>2553</v>
       </c>
       <c r="G23" s="4" t="n">
+        <v>2553</v>
+      </c>
+      <c r="H23" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="I23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="4" t="n">
         <v>2932.59499326</v>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>Get news</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>SMUSE_i_W144 == 1</t>
         </is>
@@ -19730,22 +20090,37 @@
         <v>2556</v>
       </c>
       <c r="G24" s="4" t="n">
+        <v>2556</v>
+      </c>
+      <c r="H24" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="I24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="4" t="n">
         <v>2935.07266706</v>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Keep up with politics or political issues</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>SMUSE_i_W144 == 1</t>
         </is>
@@ -19779,22 +20154,37 @@
         <v>2555</v>
       </c>
       <c r="G25" s="4" t="n">
+        <v>2555</v>
+      </c>
+      <c r="H25" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H25" s="4" t="n">
+      <c r="I25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="4" t="n">
         <v>2936.10166492</v>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>Keep up with sports or pop culture</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="P25" s="4" t="inlineStr">
         <is>
           <t>SMUSE_i_W144 == 1</t>
         </is>
@@ -19828,22 +20218,37 @@
         <v>2555</v>
       </c>
       <c r="G26" s="4" t="n">
+        <v>2555</v>
+      </c>
+      <c r="H26" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H26" s="4" t="n">
+      <c r="I26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4" t="n">
         <v>2934.52357</v>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>Entertainment</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="P26" s="4" t="inlineStr">
         <is>
           <t>SMUSE_i_W144 == 1</t>
         </is>
@@ -19877,22 +20282,37 @@
         <v>2552</v>
       </c>
       <c r="G27" s="4" t="n">
+        <v>2552</v>
+      </c>
+      <c r="H27" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H27" s="4" t="n">
+      <c r="I27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="4" t="n">
         <v>2934.20007637</v>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>Keep up with friends and family</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="P27" s="4" t="inlineStr">
         <is>
           <t>SMUSE_i_W144 == 1</t>
         </is>
@@ -19926,22 +20346,37 @@
         <v>2555</v>
       </c>
       <c r="G28" s="4" t="n">
+        <v>2555</v>
+      </c>
+      <c r="H28" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H28" s="4" t="n">
+      <c r="I28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="4" t="n">
         <v>2935.30407014</v>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>Connect with others who share your interests</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="P28" s="4" t="inlineStr">
         <is>
           <t>SMUSE_i_W144 == 1</t>
         </is>
@@ -19975,29 +20410,44 @@
         <v>2553</v>
       </c>
       <c r="G29" s="4" t="n">
+        <v>2553</v>
+      </c>
+      <c r="H29" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H29" s="4" t="n">
+      <c r="I29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="4" t="n">
         <v>2932.86439243</v>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="O29" s="4" t="inlineStr">
         <is>
           <t>Look at product reviews or recommendations</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="P29" s="4" t="inlineStr">
         <is>
           <t>SMUSE_i_W144 == 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K29"/>
+  <autoFilter ref="A1:P29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>